<commit_message>
Remove Traceability sheet from Excel report
</commit_message>
<xml_diff>
--- a/docs/SauceDemo_Automation_Test_Report.xlsx
+++ b/docs/SauceDemo_Automation_Test_Report.xlsx
@@ -12,7 +12,6 @@
     <sheet name="Test Cases" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Test Execution" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Defect Report" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Traceability" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Test Cases'!$A$1:$P$223</definedName>
@@ -824,6 +823,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="36">
       <c r="A4" s="39" t="inlineStr">
         <is>
@@ -966,6 +966,7 @@
       <c r="D13" s="42" t="n"/>
       <c r="E13" s="43" t="n"/>
     </row>
+    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="36">
       <c r="A15" s="39" t="inlineStr">
         <is>
@@ -1036,6 +1037,7 @@
       <c r="D20" s="42" t="n"/>
       <c r="E20" s="43" t="n"/>
     </row>
+    <row r="21"/>
     <row r="22" ht="15" customHeight="1" s="36">
       <c r="A22" s="39" t="inlineStr">
         <is>
@@ -1183,6 +1185,7 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
     <row r="37" ht="15" customHeight="1" s="36">
       <c r="A37" s="39" t="inlineStr">
         <is>
@@ -1588,6 +1591,7 @@
         <v/>
       </c>
     </row>
+    <row r="49"/>
     <row r="50" ht="15" customHeight="1" s="36">
       <c r="A50" s="39" t="inlineStr">
         <is>
@@ -1602,7 +1606,7 @@
         </is>
       </c>
       <c r="B51" s="49">
-        <f>COUNTIF(Traceability!$D$2:$D$16,"Covered*")</f>
+        <f>SUMPRODUCT(('Test Execution'!$N$2:$N$200&lt;&gt;"-")*('Test Execution'!$N$2:$N$200&lt;&gt;"")/COUNTIF('Test Execution'!$N$2:$N$200,'Test Execution'!$N$2:$N$200&amp;""))</f>
         <v/>
       </c>
     </row>
@@ -18905,745 +18909,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <tabColor rgb="FF217346"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:E28"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="11" customWidth="1" style="35" min="1" max="1"/>
-    <col width="42" customWidth="1" style="35" min="2" max="2"/>
-    <col width="26" customWidth="1" style="35" min="3" max="3"/>
-    <col width="24" customWidth="1" style="35" min="4" max="4"/>
-    <col width="26" customWidth="1" style="35" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1" s="36">
-      <c r="A1" s="45" t="inlineStr">
-        <is>
-          <t>Manual TC</t>
-        </is>
-      </c>
-      <c r="B1" s="45" t="inlineStr">
-        <is>
-          <t>Manual Scenario</t>
-        </is>
-      </c>
-      <c r="C1" s="45" t="inlineStr">
-        <is>
-          <t>Automation TC(s)</t>
-        </is>
-      </c>
-      <c r="D1" s="45" t="inlineStr">
-        <is>
-          <t>Coverage</t>
-        </is>
-      </c>
-      <c r="E1" s="45" t="inlineStr">
-        <is>
-          <t>Linked Bug(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="36">
-      <c r="A2" s="59" t="inlineStr">
-        <is>
-          <t>TC-001</t>
-        </is>
-      </c>
-      <c r="B2" s="60" t="inlineStr">
-        <is>
-          <t>Problem User Checkout Flow</t>
-        </is>
-      </c>
-      <c r="C2" s="60" t="inlineStr">
-        <is>
-          <t>AUT-016</t>
-        </is>
-      </c>
-      <c r="D2" s="59" t="inlineStr">
-        <is>
-          <t>Covered</t>
-        </is>
-      </c>
-      <c r="E2" s="60" t="inlineStr">
-        <is>
-          <t>BUG-001</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="36">
-      <c r="A3" s="49" t="inlineStr">
-        <is>
-          <t>TC-002</t>
-        </is>
-      </c>
-      <c r="B3" s="41" t="inlineStr">
-        <is>
-          <t>Reset App State after adding products</t>
-        </is>
-      </c>
-      <c r="C3" s="41" t="inlineStr">
-        <is>
-          <t>AUT-023</t>
-        </is>
-      </c>
-      <c r="D3" s="49" t="inlineStr">
-        <is>
-          <t>Covered</t>
-        </is>
-      </c>
-      <c r="E3" s="41" t="inlineStr">
-        <is>
-          <t>BUG-008</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="36">
-      <c r="A4" s="59" t="inlineStr">
-        <is>
-          <t>TC-003</t>
-        </is>
-      </c>
-      <c r="B4" s="60" t="inlineStr">
-        <is>
-          <t>Checkout with empty cart</t>
-        </is>
-      </c>
-      <c r="C4" s="60" t="inlineStr">
-        <is>
-          <t>AUT-024</t>
-        </is>
-      </c>
-      <c r="D4" s="59" t="inlineStr">
-        <is>
-          <t>Covered</t>
-        </is>
-      </c>
-      <c r="E4" s="60" t="inlineStr">
-        <is>
-          <t>BUG-009</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="36">
-      <c r="A5" s="49" t="inlineStr">
-        <is>
-          <t>TC-004</t>
-        </is>
-      </c>
-      <c r="B5" s="41" t="inlineStr">
-        <is>
-          <t>Error User Checkout Completion</t>
-        </is>
-      </c>
-      <c r="C5" s="41" t="inlineStr">
-        <is>
-          <t>AUT-025</t>
-        </is>
-      </c>
-      <c r="D5" s="49" t="inlineStr">
-        <is>
-          <t>Covered</t>
-        </is>
-      </c>
-      <c r="E5" s="41" t="inlineStr">
-        <is>
-          <t>BUG-010</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="36">
-      <c r="A6" s="59" t="inlineStr">
-        <is>
-          <t>TC-005</t>
-        </is>
-      </c>
-      <c r="B6" s="60" t="inlineStr">
-        <is>
-          <t>Visual User Product Display Accuracy</t>
-        </is>
-      </c>
-      <c r="C6" s="60" t="inlineStr">
-        <is>
-          <t>AUT-027, AUT-028, AUT-029</t>
-        </is>
-      </c>
-      <c r="D6" s="59" t="inlineStr">
-        <is>
-          <t>Covered (split into 3 tests)</t>
-        </is>
-      </c>
-      <c r="E6" s="60" t="inlineStr">
-        <is>
-          <t>BUG-011, BUG-012, BUG-013</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="36">
-      <c r="A7" s="49" t="inlineStr">
-        <is>
-          <t>TC-006</t>
-        </is>
-      </c>
-      <c r="B7" s="41" t="inlineStr">
-        <is>
-          <t>Cart Persistence Across Different User Logins</t>
-        </is>
-      </c>
-      <c r="C7" s="41" t="inlineStr">
-        <is>
-          <t>AUT-031</t>
-        </is>
-      </c>
-      <c r="D7" s="49" t="inlineStr">
-        <is>
-          <t>Covered</t>
-        </is>
-      </c>
-      <c r="E7" s="41" t="inlineStr">
-        <is>
-          <t>BUG-014</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="36">
-      <c r="A8" s="59" t="inlineStr">
-        <is>
-          <t>TC-007</t>
-        </is>
-      </c>
-      <c r="B8" s="60" t="inlineStr">
-        <is>
-          <t>Dynamic Catalog Menu Feature</t>
-        </is>
-      </c>
-      <c r="C8" s="60" t="inlineStr">
-        <is>
-          <t>AUT-032</t>
-        </is>
-      </c>
-      <c r="D8" s="59" t="inlineStr">
-        <is>
-          <t>Covered</t>
-        </is>
-      </c>
-      <c r="E8" s="60" t="inlineStr">
-        <is>
-          <t>BUG-015</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="36">
-      <c r="A9" s="49" t="inlineStr">
-        <is>
-          <t>TC-008</t>
-        </is>
-      </c>
-      <c r="B9" s="41" t="inlineStr">
-        <is>
-          <t>Problem User - Fleece Jacket Product Details</t>
-        </is>
-      </c>
-      <c r="C9" s="41" t="inlineStr">
-        <is>
-          <t>AUT-022</t>
-        </is>
-      </c>
-      <c r="D9" s="49" t="inlineStr">
-        <is>
-          <t>Covered</t>
-        </is>
-      </c>
-      <c r="E9" s="41" t="inlineStr">
-        <is>
-          <t>BUG-016</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="36">
-      <c r="A10" s="59" t="inlineStr">
-        <is>
-          <t>TC-009</t>
-        </is>
-      </c>
-      <c r="B10" s="60" t="inlineStr">
-        <is>
-          <t>Error User - Product Sorting</t>
-        </is>
-      </c>
-      <c r="C10" s="60" t="inlineStr">
-        <is>
-          <t>AUT-026</t>
-        </is>
-      </c>
-      <c r="D10" s="59" t="inlineStr">
-        <is>
-          <t>Covered</t>
-        </is>
-      </c>
-      <c r="E10" s="60" t="inlineStr">
-        <is>
-          <t>BUG-017</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="36">
-      <c r="A11" s="49" t="inlineStr">
-        <is>
-          <t>TC-010</t>
-        </is>
-      </c>
-      <c r="B11" s="41" t="inlineStr">
-        <is>
-          <t>Visual User - Price Sorting</t>
-        </is>
-      </c>
-      <c r="C11" s="41" t="inlineStr">
-        <is>
-          <t>AUT-030</t>
-        </is>
-      </c>
-      <c r="D11" s="49" t="inlineStr">
-        <is>
-          <t>Covered</t>
-        </is>
-      </c>
-      <c r="E11" s="41" t="inlineStr">
-        <is>
-          <t>BUG-018</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="36">
-      <c r="A12" s="59" t="inlineStr">
-        <is>
-          <t>TC-011</t>
-        </is>
-      </c>
-      <c r="B12" s="60" t="inlineStr">
-        <is>
-          <t>Successful Login to Checkout</t>
-        </is>
-      </c>
-      <c r="C12" s="60" t="inlineStr">
-        <is>
-          <t>AUT-008</t>
-        </is>
-      </c>
-      <c r="D12" s="59" t="inlineStr">
-        <is>
-          <t>Covered</t>
-        </is>
-      </c>
-      <c r="E12" s="60" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="36">
-      <c r="A13" s="49" t="inlineStr">
-        <is>
-          <t>TC-012</t>
-        </is>
-      </c>
-      <c r="B13" s="41" t="inlineStr">
-        <is>
-          <t>Checkout with missing required information</t>
-        </is>
-      </c>
-      <c r="C13" s="41" t="inlineStr">
-        <is>
-          <t>AUT-012</t>
-        </is>
-      </c>
-      <c r="D13" s="49" t="inlineStr">
-        <is>
-          <t>Covered</t>
-        </is>
-      </c>
-      <c r="E13" s="41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="36">
-      <c r="A14" s="59" t="inlineStr">
-        <is>
-          <t>TC-013</t>
-        </is>
-      </c>
-      <c r="B14" s="60" t="inlineStr">
-        <is>
-          <t>Login with locked-out user</t>
-        </is>
-      </c>
-      <c r="C14" s="60" t="inlineStr">
-        <is>
-          <t>AUT-003</t>
-        </is>
-      </c>
-      <c r="D14" s="59" t="inlineStr">
-        <is>
-          <t>Covered</t>
-        </is>
-      </c>
-      <c r="E14" s="60" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="36">
-      <c r="A15" s="49" t="inlineStr">
-        <is>
-          <t>TC-014</t>
-        </is>
-      </c>
-      <c r="B15" s="41" t="inlineStr">
-        <is>
-          <t>Remove Product Before Checkout</t>
-        </is>
-      </c>
-      <c r="C15" s="41" t="inlineStr">
-        <is>
-          <t>AUT-009</t>
-        </is>
-      </c>
-      <c r="D15" s="49" t="inlineStr">
-        <is>
-          <t>Covered</t>
-        </is>
-      </c>
-      <c r="E15" s="41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="36">
-      <c r="A16" s="59" t="inlineStr">
-        <is>
-          <t>TC-015</t>
-        </is>
-      </c>
-      <c r="B16" s="60" t="inlineStr">
-        <is>
-          <t>Checkout with Empty Cart</t>
-        </is>
-      </c>
-      <c r="C16" s="60" t="inlineStr">
-        <is>
-          <t>AUT-015</t>
-        </is>
-      </c>
-      <c r="D16" s="59" t="inlineStr">
-        <is>
-          <t>Covered</t>
-        </is>
-      </c>
-      <c r="E16" s="60" t="inlineStr">
-        <is>
-          <t>BUG-009</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18" ht="15" customHeight="1" s="36">
-      <c r="A18" s="39" t="inlineStr">
-        <is>
-          <t>Automation-only Test Cases (extensions)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1" s="36">
-      <c r="A19" s="45" t="inlineStr">
-        <is>
-          <t>Automation TC</t>
-        </is>
-      </c>
-      <c r="B19" s="45" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="C19" s="45" t="inlineStr">
-        <is>
-          <t>Suite ID</t>
-        </is>
-      </c>
-      <c r="D19" s="45" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="E19" s="45" t="inlineStr">
-        <is>
-          <t>Linked Bug</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="36">
-      <c r="A20" s="59" t="inlineStr">
-        <is>
-          <t>AUT-001</t>
-        </is>
-      </c>
-      <c r="B20" s="60" t="inlineStr">
-        <is>
-          <t>Site opens with correct title</t>
-        </is>
-      </c>
-      <c r="C20" s="59" t="inlineStr">
-        <is>
-          <t>TS-01</t>
-        </is>
-      </c>
-      <c r="D20" s="59" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="E20" s="59" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="36">
-      <c r="A21" s="59" t="inlineStr">
-        <is>
-          <t>AUT-004</t>
-        </is>
-      </c>
-      <c r="B21" s="60" t="inlineStr">
-        <is>
-          <t>Login with invalid password</t>
-        </is>
-      </c>
-      <c r="C21" s="59" t="inlineStr">
-        <is>
-          <t>TS-02</t>
-        </is>
-      </c>
-      <c r="D21" s="59" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="E21" s="59" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="36">
-      <c r="A22" s="49" t="inlineStr">
-        <is>
-          <t>AUT-007</t>
-        </is>
-      </c>
-      <c r="B22" s="41" t="inlineStr">
-        <is>
-          <t>Data-driven login for all accepted users</t>
-        </is>
-      </c>
-      <c r="C22" s="49" t="inlineStr">
-        <is>
-          <t>TS-02</t>
-        </is>
-      </c>
-      <c r="D22" s="49" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="E22" s="49" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="36">
-      <c r="A23" s="59" t="inlineStr">
-        <is>
-          <t>AUT-010</t>
-        </is>
-      </c>
-      <c r="B23" s="60" t="inlineStr">
-        <is>
-          <t>Cart total calculation with multiple items</t>
-        </is>
-      </c>
-      <c r="C23" s="59" t="inlineStr">
-        <is>
-          <t>TS-03</t>
-        </is>
-      </c>
-      <c r="D23" s="59" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="E23" s="59" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="36">
-      <c r="A24" s="49" t="inlineStr">
-        <is>
-          <t>AUT-011</t>
-        </is>
-      </c>
-      <c r="B24" s="41" t="inlineStr">
-        <is>
-          <t>Product sorting options</t>
-        </is>
-      </c>
-      <c r="C24" s="49" t="inlineStr">
-        <is>
-          <t>TS-03</t>
-        </is>
-      </c>
-      <c r="D24" s="49" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="E24" s="49" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="36">
-      <c r="A25" s="59" t="inlineStr">
-        <is>
-          <t>AUT-017</t>
-        </is>
-      </c>
-      <c r="B25" s="60" t="inlineStr">
-        <is>
-          <t>Each product has its own image</t>
-        </is>
-      </c>
-      <c r="C25" s="59" t="inlineStr">
-        <is>
-          <t>TS-05</t>
-        </is>
-      </c>
-      <c r="D25" s="59" t="inlineStr">
-        <is>
-          <t>Defect</t>
-        </is>
-      </c>
-      <c r="E25" s="59" t="inlineStr">
-        <is>
-          <t>BUG-002</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15" customHeight="1" s="36">
-      <c r="A26" s="49" t="inlineStr">
-        <is>
-          <t>AUT-018</t>
-        </is>
-      </c>
-      <c r="B26" s="41" t="inlineStr">
-        <is>
-          <t>Product link opens the correct product</t>
-        </is>
-      </c>
-      <c r="C26" s="49" t="inlineStr">
-        <is>
-          <t>TS-05</t>
-        </is>
-      </c>
-      <c r="D26" s="49" t="inlineStr">
-        <is>
-          <t>Defect</t>
-        </is>
-      </c>
-      <c r="E26" s="49" t="inlineStr">
-        <is>
-          <t>BUG-003</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="36">
-      <c r="A27" s="59" t="inlineStr">
-        <is>
-          <t>AUT-019</t>
-        </is>
-      </c>
-      <c r="B27" s="60" t="inlineStr">
-        <is>
-          <t>All products can be added to cart</t>
-        </is>
-      </c>
-      <c r="C27" s="59" t="inlineStr">
-        <is>
-          <t>TS-05</t>
-        </is>
-      </c>
-      <c r="D27" s="59" t="inlineStr">
-        <is>
-          <t>Defect</t>
-        </is>
-      </c>
-      <c r="E27" s="59" t="inlineStr">
-        <is>
-          <t>BUG-004</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15" customHeight="1" s="36">
-      <c r="A28" s="59" t="inlineStr">
-        <is>
-          <t>AUT-021</t>
-        </is>
-      </c>
-      <c r="B28" s="60" t="inlineStr">
-        <is>
-          <t>Sorting changes product order</t>
-        </is>
-      </c>
-      <c r="C28" s="59" t="inlineStr">
-        <is>
-          <t>TS-05</t>
-        </is>
-      </c>
-      <c r="D28" s="59" t="inlineStr">
-        <is>
-          <t>Defect</t>
-        </is>
-      </c>
-      <c r="E28" s="59" t="inlineStr">
-        <is>
-          <t>BUG-006</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="36"/>
-    <row r="30" ht="15" customHeight="1" s="36"/>
-    <row r="31" ht="15" customHeight="1" s="36"/>
-    <row r="32" ht="15" customHeight="1" s="36"/>
-    <row r="33" ht="15" customHeight="1" s="36"/>
-    <row r="34" ht="15" customHeight="1" s="36"/>
-    <row r="35" ht="15" customHeight="1" s="36"/>
-  </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Renumber automation test case IDs to AUT-001..AUT-026
</commit_message>
<xml_diff>
--- a/docs/SauceDemo_Automation_Test_Report.xlsx
+++ b/docs/SauceDemo_Automation_Test_Report.xlsx
@@ -823,7 +823,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="36">
       <c r="A4" s="39" t="inlineStr">
         <is>
@@ -966,7 +965,6 @@
       <c r="D13" s="42" t="n"/>
       <c r="E13" s="43" t="n"/>
     </row>
-    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="36">
       <c r="A15" s="39" t="inlineStr">
         <is>
@@ -1037,7 +1035,6 @@
       <c r="D20" s="42" t="n"/>
       <c r="E20" s="43" t="n"/>
     </row>
-    <row r="21"/>
     <row r="22" ht="15" customHeight="1" s="36">
       <c r="A22" s="39" t="inlineStr">
         <is>
@@ -1185,7 +1182,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37" ht="15" customHeight="1" s="36">
       <c r="A37" s="39" t="inlineStr">
         <is>
@@ -1591,7 +1587,6 @@
         <v/>
       </c>
     </row>
-    <row r="49"/>
     <row r="50" ht="15" customHeight="1" s="36">
       <c r="A50" s="39" t="inlineStr">
         <is>
@@ -1775,7 +1770,7 @@
       </c>
       <c r="F3" s="41" t="inlineStr">
         <is>
-          <t>AUT-003, AUT-004, AUT-007</t>
+          <t>AUT-002, AUT-003, AUT-004</t>
         </is>
       </c>
       <c r="G3" s="49">
@@ -1811,7 +1806,7 @@
       </c>
       <c r="F4" s="60" t="inlineStr">
         <is>
-          <t>AUT-008, AUT-009, AUT-010, AUT-011</t>
+          <t>AUT-005, AUT-006, AUT-007, AUT-008</t>
         </is>
       </c>
       <c r="G4" s="59">
@@ -1847,7 +1842,7 @@
       </c>
       <c r="F5" s="41" t="inlineStr">
         <is>
-          <t>AUT-012, AUT-015</t>
+          <t>AUT-009, AUT-010</t>
         </is>
       </c>
       <c r="G5" s="49">
@@ -1883,7 +1878,7 @@
       </c>
       <c r="F6" s="60" t="inlineStr">
         <is>
-          <t>AUT-016, AUT-017, AUT-018, AUT-019, AUT-021, AUT-022</t>
+          <t>AUT-011, AUT-012, AUT-013, AUT-014, AUT-015, AUT-016</t>
         </is>
       </c>
       <c r="G6" s="59">
@@ -1919,7 +1914,7 @@
       </c>
       <c r="F7" s="41" t="inlineStr">
         <is>
-          <t>AUT-023, AUT-024, AUT-031</t>
+          <t>AUT-017, AUT-018, AUT-025</t>
         </is>
       </c>
       <c r="G7" s="49">
@@ -1955,7 +1950,7 @@
       </c>
       <c r="F8" s="60" t="inlineStr">
         <is>
-          <t>AUT-025, AUT-026</t>
+          <t>AUT-019, AUT-020</t>
         </is>
       </c>
       <c r="G8" s="59">
@@ -1991,7 +1986,7 @@
       </c>
       <c r="F9" s="41" t="inlineStr">
         <is>
-          <t>AUT-027, AUT-028, AUT-029, AUT-030</t>
+          <t>AUT-021, AUT-022, AUT-023, AUT-024</t>
         </is>
       </c>
       <c r="G9" s="49">
@@ -2027,7 +2022,7 @@
       </c>
       <c r="F10" s="60" t="inlineStr">
         <is>
-          <t>AUT-032</t>
+          <t>AUT-026</t>
         </is>
       </c>
       <c r="G10" s="59">
@@ -2331,7 +2326,7 @@
     <row r="4" ht="15" customHeight="1" s="36">
       <c r="A4" s="59" t="inlineStr">
         <is>
-          <t>AUT-003</t>
+          <t>AUT-002</t>
         </is>
       </c>
       <c r="B4" s="59" t="inlineStr">
@@ -2411,7 +2406,7 @@
     <row r="5" ht="15" customHeight="1" s="36">
       <c r="A5" s="59" t="inlineStr">
         <is>
-          <t>AUT-003</t>
+          <t>AUT-002</t>
         </is>
       </c>
       <c r="B5" s="59" t="inlineStr">
@@ -2491,7 +2486,7 @@
     <row r="6" ht="15" customHeight="1" s="36">
       <c r="A6" s="59" t="inlineStr">
         <is>
-          <t>AUT-003</t>
+          <t>AUT-002</t>
         </is>
       </c>
       <c r="B6" s="59" t="inlineStr">
@@ -2571,7 +2566,7 @@
     <row r="7" ht="15" customHeight="1" s="36">
       <c r="A7" s="59" t="inlineStr">
         <is>
-          <t>AUT-003</t>
+          <t>AUT-002</t>
         </is>
       </c>
       <c r="B7" s="59" t="inlineStr">
@@ -2647,7 +2642,7 @@
     <row r="8" ht="23.85" customHeight="1" s="36">
       <c r="A8" s="59" t="inlineStr">
         <is>
-          <t>AUT-003</t>
+          <t>AUT-002</t>
         </is>
       </c>
       <c r="B8" s="59" t="inlineStr">
@@ -2723,7 +2718,7 @@
     <row r="9" ht="15" customHeight="1" s="36">
       <c r="A9" s="49" t="inlineStr">
         <is>
-          <t>AUT-004</t>
+          <t>AUT-003</t>
         </is>
       </c>
       <c r="B9" s="49" t="inlineStr">
@@ -2803,7 +2798,7 @@
     <row r="10" ht="15" customHeight="1" s="36">
       <c r="A10" s="49" t="inlineStr">
         <is>
-          <t>AUT-004</t>
+          <t>AUT-003</t>
         </is>
       </c>
       <c r="B10" s="49" t="inlineStr">
@@ -2883,7 +2878,7 @@
     <row r="11" ht="15" customHeight="1" s="36">
       <c r="A11" s="49" t="inlineStr">
         <is>
-          <t>AUT-004</t>
+          <t>AUT-003</t>
         </is>
       </c>
       <c r="B11" s="49" t="inlineStr">
@@ -2963,7 +2958,7 @@
     <row r="12" ht="15" customHeight="1" s="36">
       <c r="A12" s="49" t="inlineStr">
         <is>
-          <t>AUT-004</t>
+          <t>AUT-003</t>
         </is>
       </c>
       <c r="B12" s="49" t="inlineStr">
@@ -3039,7 +3034,7 @@
     <row r="13" ht="23.85" customHeight="1" s="36">
       <c r="A13" s="49" t="inlineStr">
         <is>
-          <t>AUT-004</t>
+          <t>AUT-003</t>
         </is>
       </c>
       <c r="B13" s="49" t="inlineStr">
@@ -3115,7 +3110,7 @@
     <row r="14" ht="15" customHeight="1" s="36">
       <c r="A14" s="59" t="inlineStr">
         <is>
-          <t>AUT-007</t>
+          <t>AUT-004</t>
         </is>
       </c>
       <c r="B14" s="59" t="inlineStr">
@@ -3195,7 +3190,7 @@
     <row r="15" ht="15" customHeight="1" s="36">
       <c r="A15" s="59" t="inlineStr">
         <is>
-          <t>AUT-007</t>
+          <t>AUT-004</t>
         </is>
       </c>
       <c r="B15" s="59" t="inlineStr">
@@ -3275,7 +3270,7 @@
     <row r="16" ht="15" customHeight="1" s="36">
       <c r="A16" s="59" t="inlineStr">
         <is>
-          <t>AUT-007</t>
+          <t>AUT-004</t>
         </is>
       </c>
       <c r="B16" s="59" t="inlineStr">
@@ -3351,7 +3346,7 @@
     <row r="17" ht="15" customHeight="1" s="36">
       <c r="A17" s="59" t="inlineStr">
         <is>
-          <t>AUT-007</t>
+          <t>AUT-004</t>
         </is>
       </c>
       <c r="B17" s="59" t="inlineStr">
@@ -3427,7 +3422,7 @@
     <row r="18" ht="23.85" customHeight="1" s="36">
       <c r="A18" s="49" t="inlineStr">
         <is>
-          <t>AUT-008</t>
+          <t>AUT-005</t>
         </is>
       </c>
       <c r="B18" s="49" t="inlineStr">
@@ -3507,7 +3502,7 @@
     <row r="19" ht="15" customHeight="1" s="36">
       <c r="A19" s="49" t="inlineStr">
         <is>
-          <t>AUT-008</t>
+          <t>AUT-005</t>
         </is>
       </c>
       <c r="B19" s="49" t="inlineStr">
@@ -3587,7 +3582,7 @@
     <row r="20" ht="15" customHeight="1" s="36">
       <c r="A20" s="49" t="inlineStr">
         <is>
-          <t>AUT-008</t>
+          <t>AUT-005</t>
         </is>
       </c>
       <c r="B20" s="49" t="inlineStr">
@@ -3667,7 +3662,7 @@
     <row r="21" ht="15" customHeight="1" s="36">
       <c r="A21" s="49" t="inlineStr">
         <is>
-          <t>AUT-008</t>
+          <t>AUT-005</t>
         </is>
       </c>
       <c r="B21" s="49" t="inlineStr">
@@ -3743,7 +3738,7 @@
     <row r="22" ht="15" customHeight="1" s="36">
       <c r="A22" s="49" t="inlineStr">
         <is>
-          <t>AUT-008</t>
+          <t>AUT-005</t>
         </is>
       </c>
       <c r="B22" s="49" t="inlineStr">
@@ -3823,7 +3818,7 @@
     <row r="23" ht="15" customHeight="1" s="36">
       <c r="A23" s="49" t="inlineStr">
         <is>
-          <t>AUT-008</t>
+          <t>AUT-005</t>
         </is>
       </c>
       <c r="B23" s="49" t="inlineStr">
@@ -3899,7 +3894,7 @@
     <row r="24" ht="15" customHeight="1" s="36">
       <c r="A24" s="49" t="inlineStr">
         <is>
-          <t>AUT-008</t>
+          <t>AUT-005</t>
         </is>
       </c>
       <c r="B24" s="49" t="inlineStr">
@@ -3975,7 +3970,7 @@
     <row r="25" ht="15" customHeight="1" s="36">
       <c r="A25" s="49" t="inlineStr">
         <is>
-          <t>AUT-008</t>
+          <t>AUT-005</t>
         </is>
       </c>
       <c r="B25" s="49" t="inlineStr">
@@ -4055,7 +4050,7 @@
     <row r="26" ht="15" customHeight="1" s="36">
       <c r="A26" s="49" t="inlineStr">
         <is>
-          <t>AUT-008</t>
+          <t>AUT-005</t>
         </is>
       </c>
       <c r="B26" s="49" t="inlineStr">
@@ -4131,7 +4126,7 @@
     <row r="27" ht="15" customHeight="1" s="36">
       <c r="A27" s="49" t="inlineStr">
         <is>
-          <t>AUT-008</t>
+          <t>AUT-005</t>
         </is>
       </c>
       <c r="B27" s="49" t="inlineStr">
@@ -4207,7 +4202,7 @@
     <row r="28" ht="15" customHeight="1" s="36">
       <c r="A28" s="49" t="inlineStr">
         <is>
-          <t>AUT-008</t>
+          <t>AUT-005</t>
         </is>
       </c>
       <c r="B28" s="49" t="inlineStr">
@@ -4283,7 +4278,7 @@
     <row r="29" ht="57.45" customHeight="1" s="36">
       <c r="A29" s="59" t="inlineStr">
         <is>
-          <t>AUT-009</t>
+          <t>AUT-006</t>
         </is>
       </c>
       <c r="B29" s="59" t="inlineStr">
@@ -4363,7 +4358,7 @@
     <row r="30" ht="57.45" customHeight="1" s="36">
       <c r="A30" s="59" t="inlineStr">
         <is>
-          <t>AUT-009</t>
+          <t>AUT-006</t>
         </is>
       </c>
       <c r="B30" s="59" t="inlineStr">
@@ -4443,7 +4438,7 @@
     <row r="31" ht="57.45" customHeight="1" s="36">
       <c r="A31" s="59" t="inlineStr">
         <is>
-          <t>AUT-009</t>
+          <t>AUT-006</t>
         </is>
       </c>
       <c r="B31" s="59" t="inlineStr">
@@ -4523,7 +4518,7 @@
     <row r="32" ht="57.45" customHeight="1" s="36">
       <c r="A32" s="59" t="inlineStr">
         <is>
-          <t>AUT-009</t>
+          <t>AUT-006</t>
         </is>
       </c>
       <c r="B32" s="59" t="inlineStr">
@@ -4599,7 +4594,7 @@
     <row r="33" ht="15" customHeight="1" s="36">
       <c r="A33" s="59" t="inlineStr">
         <is>
-          <t>AUT-009</t>
+          <t>AUT-006</t>
         </is>
       </c>
       <c r="B33" s="59" t="inlineStr">
@@ -4679,7 +4674,7 @@
     <row r="34" ht="15" customHeight="1" s="36">
       <c r="A34" s="59" t="inlineStr">
         <is>
-          <t>AUT-009</t>
+          <t>AUT-006</t>
         </is>
       </c>
       <c r="B34" s="59" t="inlineStr">
@@ -4755,7 +4750,7 @@
     <row r="35" ht="15" customHeight="1" s="36">
       <c r="A35" s="59" t="inlineStr">
         <is>
-          <t>AUT-009</t>
+          <t>AUT-006</t>
         </is>
       </c>
       <c r="B35" s="59" t="inlineStr">
@@ -4835,7 +4830,7 @@
     <row r="36" ht="15" customHeight="1" s="36">
       <c r="A36" s="59" t="inlineStr">
         <is>
-          <t>AUT-009</t>
+          <t>AUT-006</t>
         </is>
       </c>
       <c r="B36" s="59" t="inlineStr">
@@ -4911,7 +4906,7 @@
     <row r="37" ht="15" customHeight="1" s="36">
       <c r="A37" s="59" t="inlineStr">
         <is>
-          <t>AUT-009</t>
+          <t>AUT-006</t>
         </is>
       </c>
       <c r="B37" s="59" t="inlineStr">
@@ -4991,7 +4986,7 @@
     <row r="38" ht="15" customHeight="1" s="36">
       <c r="A38" s="59" t="inlineStr">
         <is>
-          <t>AUT-009</t>
+          <t>AUT-006</t>
         </is>
       </c>
       <c r="B38" s="59" t="inlineStr">
@@ -5067,7 +5062,7 @@
     <row r="39" ht="15" customHeight="1" s="36">
       <c r="A39" s="59" t="inlineStr">
         <is>
-          <t>AUT-009</t>
+          <t>AUT-006</t>
         </is>
       </c>
       <c r="B39" s="59" t="inlineStr">
@@ -5143,7 +5138,7 @@
     <row r="40" ht="23.85" customHeight="1" s="36">
       <c r="A40" s="59" t="inlineStr">
         <is>
-          <t>AUT-009</t>
+          <t>AUT-006</t>
         </is>
       </c>
       <c r="B40" s="59" t="inlineStr">
@@ -5219,7 +5214,7 @@
     <row r="41" ht="15" customHeight="1" s="36">
       <c r="A41" s="49" t="inlineStr">
         <is>
-          <t>AUT-010</t>
+          <t>AUT-007</t>
         </is>
       </c>
       <c r="B41" s="49" t="inlineStr">
@@ -5299,7 +5294,7 @@
     <row r="42" ht="23.85" customHeight="1" s="36">
       <c r="A42" s="49" t="inlineStr">
         <is>
-          <t>AUT-010</t>
+          <t>AUT-007</t>
         </is>
       </c>
       <c r="B42" s="49" t="inlineStr">
@@ -5379,7 +5374,7 @@
     <row r="43" ht="15" customHeight="1" s="36">
       <c r="A43" s="49" t="inlineStr">
         <is>
-          <t>AUT-010</t>
+          <t>AUT-007</t>
         </is>
       </c>
       <c r="B43" s="49" t="inlineStr">
@@ -5459,7 +5454,7 @@
     <row r="44" ht="15" customHeight="1" s="36">
       <c r="A44" s="49" t="inlineStr">
         <is>
-          <t>AUT-010</t>
+          <t>AUT-007</t>
         </is>
       </c>
       <c r="B44" s="49" t="inlineStr">
@@ -5535,7 +5530,7 @@
     <row r="45" ht="15" customHeight="1" s="36">
       <c r="A45" s="49" t="inlineStr">
         <is>
-          <t>AUT-010</t>
+          <t>AUT-007</t>
         </is>
       </c>
       <c r="B45" s="49" t="inlineStr">
@@ -5615,7 +5610,7 @@
     <row r="46" ht="15" customHeight="1" s="36">
       <c r="A46" s="49" t="inlineStr">
         <is>
-          <t>AUT-010</t>
+          <t>AUT-007</t>
         </is>
       </c>
       <c r="B46" s="49" t="inlineStr">
@@ -5691,7 +5686,7 @@
     <row r="47" ht="15" customHeight="1" s="36">
       <c r="A47" s="49" t="inlineStr">
         <is>
-          <t>AUT-010</t>
+          <t>AUT-007</t>
         </is>
       </c>
       <c r="B47" s="49" t="inlineStr">
@@ -5771,7 +5766,7 @@
     <row r="48" ht="23.85" customHeight="1" s="36">
       <c r="A48" s="49" t="inlineStr">
         <is>
-          <t>AUT-010</t>
+          <t>AUT-007</t>
         </is>
       </c>
       <c r="B48" s="49" t="inlineStr">
@@ -5847,7 +5842,7 @@
     <row r="49" ht="15" customHeight="1" s="36">
       <c r="A49" s="49" t="inlineStr">
         <is>
-          <t>AUT-010</t>
+          <t>AUT-007</t>
         </is>
       </c>
       <c r="B49" s="49" t="inlineStr">
@@ -5927,7 +5922,7 @@
     <row r="50" ht="23.85" customHeight="1" s="36">
       <c r="A50" s="49" t="inlineStr">
         <is>
-          <t>AUT-010</t>
+          <t>AUT-007</t>
         </is>
       </c>
       <c r="B50" s="49" t="inlineStr">
@@ -6007,7 +6002,7 @@
     <row r="51" ht="15" customHeight="1" s="36">
       <c r="A51" s="49" t="inlineStr">
         <is>
-          <t>AUT-010</t>
+          <t>AUT-007</t>
         </is>
       </c>
       <c r="B51" s="49" t="inlineStr">
@@ -6087,7 +6082,7 @@
     <row r="52" ht="23.85" customHeight="1" s="36">
       <c r="A52" s="59" t="inlineStr">
         <is>
-          <t>AUT-011</t>
+          <t>AUT-008</t>
         </is>
       </c>
       <c r="B52" s="59" t="inlineStr">
@@ -6167,7 +6162,7 @@
     <row r="53" ht="15" customHeight="1" s="36">
       <c r="A53" s="59" t="inlineStr">
         <is>
-          <t>AUT-011</t>
+          <t>AUT-008</t>
         </is>
       </c>
       <c r="B53" s="59" t="inlineStr">
@@ -6247,7 +6242,7 @@
     <row r="54" ht="15" customHeight="1" s="36">
       <c r="A54" s="59" t="inlineStr">
         <is>
-          <t>AUT-011</t>
+          <t>AUT-008</t>
         </is>
       </c>
       <c r="B54" s="59" t="inlineStr">
@@ -6327,7 +6322,7 @@
     <row r="55" ht="15" customHeight="1" s="36">
       <c r="A55" s="59" t="inlineStr">
         <is>
-          <t>AUT-011</t>
+          <t>AUT-008</t>
         </is>
       </c>
       <c r="B55" s="59" t="inlineStr">
@@ -6403,7 +6398,7 @@
     <row r="56" ht="23.85" customHeight="1" s="36">
       <c r="A56" s="59" t="inlineStr">
         <is>
-          <t>AUT-011</t>
+          <t>AUT-008</t>
         </is>
       </c>
       <c r="B56" s="59" t="inlineStr">
@@ -6479,7 +6474,7 @@
     <row r="57" ht="23.85" customHeight="1" s="36">
       <c r="A57" s="59" t="inlineStr">
         <is>
-          <t>AUT-011</t>
+          <t>AUT-008</t>
         </is>
       </c>
       <c r="B57" s="59" t="inlineStr">
@@ -6555,7 +6550,7 @@
     <row r="58" ht="23.85" customHeight="1" s="36">
       <c r="A58" s="59" t="inlineStr">
         <is>
-          <t>AUT-011</t>
+          <t>AUT-008</t>
         </is>
       </c>
       <c r="B58" s="59" t="inlineStr">
@@ -6631,7 +6626,7 @@
     <row r="59" ht="23.85" customHeight="1" s="36">
       <c r="A59" s="59" t="inlineStr">
         <is>
-          <t>AUT-011</t>
+          <t>AUT-008</t>
         </is>
       </c>
       <c r="B59" s="59" t="inlineStr">
@@ -6707,7 +6702,7 @@
     <row r="60" ht="23.85" customHeight="1" s="36">
       <c r="A60" s="49" t="inlineStr">
         <is>
-          <t>AUT-012</t>
+          <t>AUT-009</t>
         </is>
       </c>
       <c r="B60" s="49" t="inlineStr">
@@ -6787,7 +6782,7 @@
     <row r="61" ht="23.85" customHeight="1" s="36">
       <c r="A61" s="49" t="inlineStr">
         <is>
-          <t>AUT-012</t>
+          <t>AUT-009</t>
         </is>
       </c>
       <c r="B61" s="49" t="inlineStr">
@@ -6867,7 +6862,7 @@
     <row r="62" ht="23.85" customHeight="1" s="36">
       <c r="A62" s="49" t="inlineStr">
         <is>
-          <t>AUT-012</t>
+          <t>AUT-009</t>
         </is>
       </c>
       <c r="B62" s="49" t="inlineStr">
@@ -6947,7 +6942,7 @@
     <row r="63" ht="23.85" customHeight="1" s="36">
       <c r="A63" s="49" t="inlineStr">
         <is>
-          <t>AUT-012</t>
+          <t>AUT-009</t>
         </is>
       </c>
       <c r="B63" s="49" t="inlineStr">
@@ -7023,7 +7018,7 @@
     <row r="64" ht="23.85" customHeight="1" s="36">
       <c r="A64" s="49" t="inlineStr">
         <is>
-          <t>AUT-012</t>
+          <t>AUT-009</t>
         </is>
       </c>
       <c r="B64" s="49" t="inlineStr">
@@ -7103,7 +7098,7 @@
     <row r="65" ht="23.85" customHeight="1" s="36">
       <c r="A65" s="49" t="inlineStr">
         <is>
-          <t>AUT-012</t>
+          <t>AUT-009</t>
         </is>
       </c>
       <c r="B65" s="49" t="inlineStr">
@@ -7179,7 +7174,7 @@
     <row r="66" ht="23.85" customHeight="1" s="36">
       <c r="A66" s="49" t="inlineStr">
         <is>
-          <t>AUT-012</t>
+          <t>AUT-009</t>
         </is>
       </c>
       <c r="B66" s="49" t="inlineStr">
@@ -7255,7 +7250,7 @@
     <row r="67" ht="15" customHeight="1" s="36">
       <c r="A67" s="49" t="inlineStr">
         <is>
-          <t>AUT-012</t>
+          <t>AUT-009</t>
         </is>
       </c>
       <c r="B67" s="49" t="inlineStr">
@@ -7335,7 +7330,7 @@
     <row r="68" ht="15" customHeight="1" s="36">
       <c r="A68" s="49" t="inlineStr">
         <is>
-          <t>AUT-012</t>
+          <t>AUT-009</t>
         </is>
       </c>
       <c r="B68" s="49" t="inlineStr">
@@ -7411,7 +7406,7 @@
     <row r="69" ht="15" customHeight="1" s="36">
       <c r="A69" s="59" t="inlineStr">
         <is>
-          <t>AUT-015</t>
+          <t>AUT-010</t>
         </is>
       </c>
       <c r="B69" s="59" t="inlineStr">
@@ -7491,7 +7486,7 @@
     <row r="70" ht="15" customHeight="1" s="36">
       <c r="A70" s="59" t="inlineStr">
         <is>
-          <t>AUT-015</t>
+          <t>AUT-010</t>
         </is>
       </c>
       <c r="B70" s="59" t="inlineStr">
@@ -7571,7 +7566,7 @@
     <row r="71" ht="15" customHeight="1" s="36">
       <c r="A71" s="59" t="inlineStr">
         <is>
-          <t>AUT-015</t>
+          <t>AUT-010</t>
         </is>
       </c>
       <c r="B71" s="59" t="inlineStr">
@@ -7651,7 +7646,7 @@
     <row r="72" ht="15" customHeight="1" s="36">
       <c r="A72" s="59" t="inlineStr">
         <is>
-          <t>AUT-015</t>
+          <t>AUT-010</t>
         </is>
       </c>
       <c r="B72" s="59" t="inlineStr">
@@ -7727,7 +7722,7 @@
     <row r="73" ht="15" customHeight="1" s="36">
       <c r="A73" s="59" t="inlineStr">
         <is>
-          <t>AUT-015</t>
+          <t>AUT-010</t>
         </is>
       </c>
       <c r="B73" s="59" t="inlineStr">
@@ -7803,7 +7798,7 @@
     <row r="74" ht="15" customHeight="1" s="36">
       <c r="A74" s="59" t="inlineStr">
         <is>
-          <t>AUT-015</t>
+          <t>AUT-010</t>
         </is>
       </c>
       <c r="B74" s="59" t="inlineStr">
@@ -7879,7 +7874,7 @@
     <row r="75" ht="15" customHeight="1" s="36">
       <c r="A75" s="49" t="inlineStr">
         <is>
-          <t>AUT-016</t>
+          <t>AUT-011</t>
         </is>
       </c>
       <c r="B75" s="49" t="inlineStr">
@@ -7959,7 +7954,7 @@
     <row r="76" ht="15" customHeight="1" s="36">
       <c r="A76" s="49" t="inlineStr">
         <is>
-          <t>AUT-016</t>
+          <t>AUT-011</t>
         </is>
       </c>
       <c r="B76" s="49" t="inlineStr">
@@ -8039,7 +8034,7 @@
     <row r="77" ht="15" customHeight="1" s="36">
       <c r="A77" s="49" t="inlineStr">
         <is>
-          <t>AUT-016</t>
+          <t>AUT-011</t>
         </is>
       </c>
       <c r="B77" s="49" t="inlineStr">
@@ -8119,7 +8114,7 @@
     <row r="78" ht="15" customHeight="1" s="36">
       <c r="A78" s="49" t="inlineStr">
         <is>
-          <t>AUT-016</t>
+          <t>AUT-011</t>
         </is>
       </c>
       <c r="B78" s="49" t="inlineStr">
@@ -8195,7 +8190,7 @@
     <row r="79" ht="15" customHeight="1" s="36">
       <c r="A79" s="49" t="inlineStr">
         <is>
-          <t>AUT-016</t>
+          <t>AUT-011</t>
         </is>
       </c>
       <c r="B79" s="49" t="inlineStr">
@@ -8275,7 +8270,7 @@
     <row r="80" ht="15" customHeight="1" s="36">
       <c r="A80" s="49" t="inlineStr">
         <is>
-          <t>AUT-016</t>
+          <t>AUT-011</t>
         </is>
       </c>
       <c r="B80" s="49" t="inlineStr">
@@ -8351,7 +8346,7 @@
     <row r="81" ht="15" customHeight="1" s="36">
       <c r="A81" s="49" t="inlineStr">
         <is>
-          <t>AUT-016</t>
+          <t>AUT-011</t>
         </is>
       </c>
       <c r="B81" s="49" t="inlineStr">
@@ -8427,7 +8422,7 @@
     <row r="82" ht="23.85" customHeight="1" s="36">
       <c r="A82" s="49" t="inlineStr">
         <is>
-          <t>AUT-016</t>
+          <t>AUT-011</t>
         </is>
       </c>
       <c r="B82" s="49" t="inlineStr">
@@ -8507,7 +8502,7 @@
     <row r="83" ht="23.85" customHeight="1" s="36">
       <c r="A83" s="49" t="inlineStr">
         <is>
-          <t>AUT-016</t>
+          <t>AUT-011</t>
         </is>
       </c>
       <c r="B83" s="49" t="inlineStr">
@@ -8587,7 +8582,7 @@
     <row r="84" ht="15" customHeight="1" s="36">
       <c r="A84" s="49" t="inlineStr">
         <is>
-          <t>AUT-016</t>
+          <t>AUT-011</t>
         </is>
       </c>
       <c r="B84" s="49" t="inlineStr">
@@ -8667,7 +8662,7 @@
     <row r="85" ht="15" customHeight="1" s="36">
       <c r="A85" s="49" t="inlineStr">
         <is>
-          <t>AUT-016</t>
+          <t>AUT-011</t>
         </is>
       </c>
       <c r="B85" s="49" t="inlineStr">
@@ -8743,7 +8738,7 @@
     <row r="86" ht="15" customHeight="1" s="36">
       <c r="A86" s="59" t="inlineStr">
         <is>
-          <t>AUT-017</t>
+          <t>AUT-012</t>
         </is>
       </c>
       <c r="B86" s="59" t="inlineStr">
@@ -8823,7 +8818,7 @@
     <row r="87" ht="15" customHeight="1" s="36">
       <c r="A87" s="59" t="inlineStr">
         <is>
-          <t>AUT-017</t>
+          <t>AUT-012</t>
         </is>
       </c>
       <c r="B87" s="59" t="inlineStr">
@@ -8903,7 +8898,7 @@
     <row r="88" ht="15" customHeight="1" s="36">
       <c r="A88" s="59" t="inlineStr">
         <is>
-          <t>AUT-017</t>
+          <t>AUT-012</t>
         </is>
       </c>
       <c r="B88" s="59" t="inlineStr">
@@ -8983,7 +8978,7 @@
     <row r="89" ht="15" customHeight="1" s="36">
       <c r="A89" s="59" t="inlineStr">
         <is>
-          <t>AUT-017</t>
+          <t>AUT-012</t>
         </is>
       </c>
       <c r="B89" s="59" t="inlineStr">
@@ -9059,7 +9054,7 @@
     <row r="90" ht="15" customHeight="1" s="36">
       <c r="A90" s="59" t="inlineStr">
         <is>
-          <t>AUT-017</t>
+          <t>AUT-012</t>
         </is>
       </c>
       <c r="B90" s="59" t="inlineStr">
@@ -9135,7 +9130,7 @@
     <row r="91" ht="23.85" customHeight="1" s="36">
       <c r="A91" s="49" t="inlineStr">
         <is>
-          <t>AUT-018</t>
+          <t>AUT-013</t>
         </is>
       </c>
       <c r="B91" s="49" t="inlineStr">
@@ -9215,7 +9210,7 @@
     <row r="92" ht="23.85" customHeight="1" s="36">
       <c r="A92" s="49" t="inlineStr">
         <is>
-          <t>AUT-018</t>
+          <t>AUT-013</t>
         </is>
       </c>
       <c r="B92" s="49" t="inlineStr">
@@ -9295,7 +9290,7 @@
     <row r="93" ht="23.85" customHeight="1" s="36">
       <c r="A93" s="49" t="inlineStr">
         <is>
-          <t>AUT-018</t>
+          <t>AUT-013</t>
         </is>
       </c>
       <c r="B93" s="49" t="inlineStr">
@@ -9375,7 +9370,7 @@
     <row r="94" ht="23.85" customHeight="1" s="36">
       <c r="A94" s="49" t="inlineStr">
         <is>
-          <t>AUT-018</t>
+          <t>AUT-013</t>
         </is>
       </c>
       <c r="B94" s="49" t="inlineStr">
@@ -9451,7 +9446,7 @@
     <row r="95" ht="23.85" customHeight="1" s="36">
       <c r="A95" s="49" t="inlineStr">
         <is>
-          <t>AUT-018</t>
+          <t>AUT-013</t>
         </is>
       </c>
       <c r="B95" s="49" t="inlineStr">
@@ -9531,7 +9526,7 @@
     <row r="96" ht="23.85" customHeight="1" s="36">
       <c r="A96" s="59" t="inlineStr">
         <is>
-          <t>AUT-019</t>
+          <t>AUT-014</t>
         </is>
       </c>
       <c r="B96" s="59" t="inlineStr">
@@ -9611,7 +9606,7 @@
     <row r="97" ht="23.85" customHeight="1" s="36">
       <c r="A97" s="59" t="inlineStr">
         <is>
-          <t>AUT-019</t>
+          <t>AUT-014</t>
         </is>
       </c>
       <c r="B97" s="59" t="inlineStr">
@@ -9691,7 +9686,7 @@
     <row r="98" ht="23.85" customHeight="1" s="36">
       <c r="A98" s="59" t="inlineStr">
         <is>
-          <t>AUT-019</t>
+          <t>AUT-014</t>
         </is>
       </c>
       <c r="B98" s="59" t="inlineStr">
@@ -9771,7 +9766,7 @@
     <row r="99" ht="23.85" customHeight="1" s="36">
       <c r="A99" s="59" t="inlineStr">
         <is>
-          <t>AUT-019</t>
+          <t>AUT-014</t>
         </is>
       </c>
       <c r="B99" s="59" t="inlineStr">
@@ -9847,7 +9842,7 @@
     <row r="100" ht="23.85" customHeight="1" s="36">
       <c r="A100" s="59" t="inlineStr">
         <is>
-          <t>AUT-019</t>
+          <t>AUT-014</t>
         </is>
       </c>
       <c r="B100" s="59" t="inlineStr">
@@ -9923,7 +9918,7 @@
     <row r="101" ht="23.85" customHeight="1" s="36">
       <c r="A101" s="59" t="inlineStr">
         <is>
-          <t>AUT-021</t>
+          <t>AUT-015</t>
         </is>
       </c>
       <c r="B101" s="59" t="inlineStr">
@@ -10003,7 +9998,7 @@
     <row r="102" ht="23.85" customHeight="1" s="36">
       <c r="A102" s="59" t="inlineStr">
         <is>
-          <t>AUT-021</t>
+          <t>AUT-015</t>
         </is>
       </c>
       <c r="B102" s="59" t="inlineStr">
@@ -10083,7 +10078,7 @@
     <row r="103" ht="23.85" customHeight="1" s="36">
       <c r="A103" s="59" t="inlineStr">
         <is>
-          <t>AUT-021</t>
+          <t>AUT-015</t>
         </is>
       </c>
       <c r="B103" s="59" t="inlineStr">
@@ -10163,7 +10158,7 @@
     <row r="104" ht="23.85" customHeight="1" s="36">
       <c r="A104" s="59" t="inlineStr">
         <is>
-          <t>AUT-021</t>
+          <t>AUT-015</t>
         </is>
       </c>
       <c r="B104" s="59" t="inlineStr">
@@ -10239,7 +10234,7 @@
     <row r="105" ht="23.85" customHeight="1" s="36">
       <c r="A105" s="59" t="inlineStr">
         <is>
-          <t>AUT-021</t>
+          <t>AUT-015</t>
         </is>
       </c>
       <c r="B105" s="59" t="inlineStr">
@@ -10315,7 +10310,7 @@
     <row r="106" ht="23.85" customHeight="1" s="36">
       <c r="A106" s="49" t="inlineStr">
         <is>
-          <t>AUT-022</t>
+          <t>AUT-016</t>
         </is>
       </c>
       <c r="B106" s="49" t="inlineStr">
@@ -10395,7 +10390,7 @@
     <row r="107" ht="23.85" customHeight="1" s="36">
       <c r="A107" s="49" t="inlineStr">
         <is>
-          <t>AUT-022</t>
+          <t>AUT-016</t>
         </is>
       </c>
       <c r="B107" s="49" t="inlineStr">
@@ -10475,7 +10470,7 @@
     <row r="108" ht="15" customHeight="1" s="36">
       <c r="A108" s="49" t="inlineStr">
         <is>
-          <t>AUT-022</t>
+          <t>AUT-016</t>
         </is>
       </c>
       <c r="B108" s="49" t="inlineStr">
@@ -10555,7 +10550,7 @@
     <row r="109" ht="15" customHeight="1" s="36">
       <c r="A109" s="49" t="inlineStr">
         <is>
-          <t>AUT-022</t>
+          <t>AUT-016</t>
         </is>
       </c>
       <c r="B109" s="49" t="inlineStr">
@@ -10631,7 +10626,7 @@
     <row r="110" ht="15" customHeight="1" s="36">
       <c r="A110" s="49" t="inlineStr">
         <is>
-          <t>AUT-022</t>
+          <t>AUT-016</t>
         </is>
       </c>
       <c r="B110" s="49" t="inlineStr">
@@ -10711,7 +10706,7 @@
     <row r="111" ht="15" customHeight="1" s="36">
       <c r="A111" s="59" t="inlineStr">
         <is>
-          <t>AUT-023</t>
+          <t>AUT-017</t>
         </is>
       </c>
       <c r="B111" s="59" t="inlineStr">
@@ -10791,7 +10786,7 @@
     <row r="112" ht="15" customHeight="1" s="36">
       <c r="A112" s="59" t="inlineStr">
         <is>
-          <t>AUT-023</t>
+          <t>AUT-017</t>
         </is>
       </c>
       <c r="B112" s="59" t="inlineStr">
@@ -10871,7 +10866,7 @@
     <row r="113" ht="15" customHeight="1" s="36">
       <c r="A113" s="59" t="inlineStr">
         <is>
-          <t>AUT-023</t>
+          <t>AUT-017</t>
         </is>
       </c>
       <c r="B113" s="59" t="inlineStr">
@@ -10951,7 +10946,7 @@
     <row r="114" ht="15" customHeight="1" s="36">
       <c r="A114" s="59" t="inlineStr">
         <is>
-          <t>AUT-023</t>
+          <t>AUT-017</t>
         </is>
       </c>
       <c r="B114" s="59" t="inlineStr">
@@ -11027,7 +11022,7 @@
     <row r="115" ht="15" customHeight="1" s="36">
       <c r="A115" s="59" t="inlineStr">
         <is>
-          <t>AUT-023</t>
+          <t>AUT-017</t>
         </is>
       </c>
       <c r="B115" s="59" t="inlineStr">
@@ -11107,7 +11102,7 @@
     <row r="116" ht="23.85" customHeight="1" s="36">
       <c r="A116" s="59" t="inlineStr">
         <is>
-          <t>AUT-023</t>
+          <t>AUT-017</t>
         </is>
       </c>
       <c r="B116" s="59" t="inlineStr">
@@ -11183,7 +11178,7 @@
     <row r="117" ht="15" customHeight="1" s="36">
       <c r="A117" s="59" t="inlineStr">
         <is>
-          <t>AUT-023</t>
+          <t>AUT-017</t>
         </is>
       </c>
       <c r="B117" s="59" t="inlineStr">
@@ -11259,7 +11254,7 @@
     <row r="118" ht="15" customHeight="1" s="36">
       <c r="A118" s="49" t="inlineStr">
         <is>
-          <t>AUT-024</t>
+          <t>AUT-018</t>
         </is>
       </c>
       <c r="B118" s="49" t="inlineStr">
@@ -11339,7 +11334,7 @@
     <row r="119" ht="15" customHeight="1" s="36">
       <c r="A119" s="49" t="inlineStr">
         <is>
-          <t>AUT-024</t>
+          <t>AUT-018</t>
         </is>
       </c>
       <c r="B119" s="49" t="inlineStr">
@@ -11419,7 +11414,7 @@
     <row r="120" ht="15" customHeight="1" s="36">
       <c r="A120" s="49" t="inlineStr">
         <is>
-          <t>AUT-024</t>
+          <t>AUT-018</t>
         </is>
       </c>
       <c r="B120" s="49" t="inlineStr">
@@ -11499,7 +11494,7 @@
     <row r="121" ht="15" customHeight="1" s="36">
       <c r="A121" s="49" t="inlineStr">
         <is>
-          <t>AUT-024</t>
+          <t>AUT-018</t>
         </is>
       </c>
       <c r="B121" s="49" t="inlineStr">
@@ -11575,7 +11570,7 @@
     <row r="122" ht="15" customHeight="1" s="36">
       <c r="A122" s="49" t="inlineStr">
         <is>
-          <t>AUT-024</t>
+          <t>AUT-018</t>
         </is>
       </c>
       <c r="B122" s="49" t="inlineStr">
@@ -11651,7 +11646,7 @@
     <row r="123" ht="15" customHeight="1" s="36">
       <c r="A123" s="49" t="inlineStr">
         <is>
-          <t>AUT-024</t>
+          <t>AUT-018</t>
         </is>
       </c>
       <c r="B123" s="49" t="inlineStr">
@@ -11727,7 +11722,7 @@
     <row r="124" ht="23.85" customHeight="1" s="36">
       <c r="A124" s="49" t="inlineStr">
         <is>
-          <t>AUT-024</t>
+          <t>AUT-018</t>
         </is>
       </c>
       <c r="B124" s="49" t="inlineStr">
@@ -11807,7 +11802,7 @@
     <row r="125" ht="23.85" customHeight="1" s="36">
       <c r="A125" s="49" t="inlineStr">
         <is>
-          <t>AUT-024</t>
+          <t>AUT-018</t>
         </is>
       </c>
       <c r="B125" s="49" t="inlineStr">
@@ -11883,7 +11878,7 @@
     <row r="126" ht="23.85" customHeight="1" s="36">
       <c r="A126" s="49" t="inlineStr">
         <is>
-          <t>AUT-024</t>
+          <t>AUT-018</t>
         </is>
       </c>
       <c r="B126" s="49" t="inlineStr">
@@ -11959,7 +11954,7 @@
     <row r="127" ht="23.85" customHeight="1" s="36">
       <c r="A127" s="59" t="inlineStr">
         <is>
-          <t>AUT-025</t>
+          <t>AUT-019</t>
         </is>
       </c>
       <c r="B127" s="59" t="inlineStr">
@@ -12039,7 +12034,7 @@
     <row r="128" ht="23.85" customHeight="1" s="36">
       <c r="A128" s="59" t="inlineStr">
         <is>
-          <t>AUT-025</t>
+          <t>AUT-019</t>
         </is>
       </c>
       <c r="B128" s="59" t="inlineStr">
@@ -12119,7 +12114,7 @@
     <row r="129" ht="15" customHeight="1" s="36">
       <c r="A129" s="59" t="inlineStr">
         <is>
-          <t>AUT-025</t>
+          <t>AUT-019</t>
         </is>
       </c>
       <c r="B129" s="59" t="inlineStr">
@@ -12199,7 +12194,7 @@
     <row r="130" ht="15" customHeight="1" s="36">
       <c r="A130" s="59" t="inlineStr">
         <is>
-          <t>AUT-025</t>
+          <t>AUT-019</t>
         </is>
       </c>
       <c r="B130" s="59" t="inlineStr">
@@ -12275,7 +12270,7 @@
     <row r="131" ht="15" customHeight="1" s="36">
       <c r="A131" s="59" t="inlineStr">
         <is>
-          <t>AUT-025</t>
+          <t>AUT-019</t>
         </is>
       </c>
       <c r="B131" s="59" t="inlineStr">
@@ -12355,7 +12350,7 @@
     <row r="132" ht="15" customHeight="1" s="36">
       <c r="A132" s="59" t="inlineStr">
         <is>
-          <t>AUT-025</t>
+          <t>AUT-019</t>
         </is>
       </c>
       <c r="B132" s="59" t="inlineStr">
@@ -12431,7 +12426,7 @@
     <row r="133" ht="15" customHeight="1" s="36">
       <c r="A133" s="59" t="inlineStr">
         <is>
-          <t>AUT-025</t>
+          <t>AUT-019</t>
         </is>
       </c>
       <c r="B133" s="59" t="inlineStr">
@@ -12507,7 +12502,7 @@
     <row r="134" ht="15" customHeight="1" s="36">
       <c r="A134" s="59" t="inlineStr">
         <is>
-          <t>AUT-025</t>
+          <t>AUT-019</t>
         </is>
       </c>
       <c r="B134" s="59" t="inlineStr">
@@ -12587,7 +12582,7 @@
     <row r="135" ht="15" customHeight="1" s="36">
       <c r="A135" s="59" t="inlineStr">
         <is>
-          <t>AUT-025</t>
+          <t>AUT-019</t>
         </is>
       </c>
       <c r="B135" s="59" t="inlineStr">
@@ -12663,7 +12658,7 @@
     <row r="136" ht="15" customHeight="1" s="36">
       <c r="A136" s="59" t="inlineStr">
         <is>
-          <t>AUT-025</t>
+          <t>AUT-019</t>
         </is>
       </c>
       <c r="B136" s="59" t="inlineStr">
@@ -12739,7 +12734,7 @@
     <row r="137" ht="15" customHeight="1" s="36">
       <c r="A137" s="59" t="inlineStr">
         <is>
-          <t>AUT-025</t>
+          <t>AUT-019</t>
         </is>
       </c>
       <c r="B137" s="59" t="inlineStr">
@@ -12815,7 +12810,7 @@
     <row r="138" ht="15" customHeight="1" s="36">
       <c r="A138" s="49" t="inlineStr">
         <is>
-          <t>AUT-026</t>
+          <t>AUT-020</t>
         </is>
       </c>
       <c r="B138" s="49" t="inlineStr">
@@ -12895,7 +12890,7 @@
     <row r="139" ht="15" customHeight="1" s="36">
       <c r="A139" s="49" t="inlineStr">
         <is>
-          <t>AUT-026</t>
+          <t>AUT-020</t>
         </is>
       </c>
       <c r="B139" s="49" t="inlineStr">
@@ -12975,7 +12970,7 @@
     <row r="140" ht="15" customHeight="1" s="36">
       <c r="A140" s="49" t="inlineStr">
         <is>
-          <t>AUT-026</t>
+          <t>AUT-020</t>
         </is>
       </c>
       <c r="B140" s="49" t="inlineStr">
@@ -13055,7 +13050,7 @@
     <row r="141" ht="15" customHeight="1" s="36">
       <c r="A141" s="49" t="inlineStr">
         <is>
-          <t>AUT-026</t>
+          <t>AUT-020</t>
         </is>
       </c>
       <c r="B141" s="49" t="inlineStr">
@@ -13131,7 +13126,7 @@
     <row r="142" ht="15" customHeight="1" s="36">
       <c r="A142" s="49" t="inlineStr">
         <is>
-          <t>AUT-026</t>
+          <t>AUT-020</t>
         </is>
       </c>
       <c r="B142" s="49" t="inlineStr">
@@ -13207,7 +13202,7 @@
     <row r="143" ht="15" customHeight="1" s="36">
       <c r="A143" s="59" t="inlineStr">
         <is>
-          <t>AUT-027</t>
+          <t>AUT-021</t>
         </is>
       </c>
       <c r="B143" s="59" t="inlineStr">
@@ -13287,7 +13282,7 @@
     <row r="144" ht="15" customHeight="1" s="36">
       <c r="A144" s="59" t="inlineStr">
         <is>
-          <t>AUT-027</t>
+          <t>AUT-021</t>
         </is>
       </c>
       <c r="B144" s="59" t="inlineStr">
@@ -13367,7 +13362,7 @@
     <row r="145" ht="15" customHeight="1" s="36">
       <c r="A145" s="59" t="inlineStr">
         <is>
-          <t>AUT-027</t>
+          <t>AUT-021</t>
         </is>
       </c>
       <c r="B145" s="59" t="inlineStr">
@@ -13447,7 +13442,7 @@
     <row r="146" ht="15" customHeight="1" s="36">
       <c r="A146" s="59" t="inlineStr">
         <is>
-          <t>AUT-027</t>
+          <t>AUT-021</t>
         </is>
       </c>
       <c r="B146" s="59" t="inlineStr">
@@ -13523,7 +13518,7 @@
     <row r="147" ht="15" customHeight="1" s="36">
       <c r="A147" s="59" t="inlineStr">
         <is>
-          <t>AUT-027</t>
+          <t>AUT-021</t>
         </is>
       </c>
       <c r="B147" s="59" t="inlineStr">
@@ -13603,7 +13598,7 @@
     <row r="148" ht="15" customHeight="1" s="36">
       <c r="A148" s="49" t="inlineStr">
         <is>
-          <t>AUT-028</t>
+          <t>AUT-022</t>
         </is>
       </c>
       <c r="B148" s="49" t="inlineStr">
@@ -13683,7 +13678,7 @@
     <row r="149" ht="23.85" customHeight="1" s="36">
       <c r="A149" s="49" t="inlineStr">
         <is>
-          <t>AUT-028</t>
+          <t>AUT-022</t>
         </is>
       </c>
       <c r="B149" s="49" t="inlineStr">
@@ -13763,7 +13758,7 @@
     <row r="150" ht="23.85" customHeight="1" s="36">
       <c r="A150" s="49" t="inlineStr">
         <is>
-          <t>AUT-028</t>
+          <t>AUT-022</t>
         </is>
       </c>
       <c r="B150" s="49" t="inlineStr">
@@ -13843,7 +13838,7 @@
     <row r="151" ht="23.85" customHeight="1" s="36">
       <c r="A151" s="49" t="inlineStr">
         <is>
-          <t>AUT-028</t>
+          <t>AUT-022</t>
         </is>
       </c>
       <c r="B151" s="49" t="inlineStr">
@@ -13919,7 +13914,7 @@
     <row r="152" ht="23.85" customHeight="1" s="36">
       <c r="A152" s="49" t="inlineStr">
         <is>
-          <t>AUT-028</t>
+          <t>AUT-022</t>
         </is>
       </c>
       <c r="B152" s="49" t="inlineStr">
@@ -13995,7 +13990,7 @@
     <row r="153" ht="23.85" customHeight="1" s="36">
       <c r="A153" s="59" t="inlineStr">
         <is>
-          <t>AUT-029</t>
+          <t>AUT-023</t>
         </is>
       </c>
       <c r="B153" s="59" t="inlineStr">
@@ -14075,7 +14070,7 @@
     <row r="154" ht="23.85" customHeight="1" s="36">
       <c r="A154" s="59" t="inlineStr">
         <is>
-          <t>AUT-029</t>
+          <t>AUT-023</t>
         </is>
       </c>
       <c r="B154" s="59" t="inlineStr">
@@ -14155,7 +14150,7 @@
     <row r="155" ht="23.85" customHeight="1" s="36">
       <c r="A155" s="59" t="inlineStr">
         <is>
-          <t>AUT-029</t>
+          <t>AUT-023</t>
         </is>
       </c>
       <c r="B155" s="59" t="inlineStr">
@@ -14235,7 +14230,7 @@
     <row r="156" ht="23.85" customHeight="1" s="36">
       <c r="A156" s="59" t="inlineStr">
         <is>
-          <t>AUT-029</t>
+          <t>AUT-023</t>
         </is>
       </c>
       <c r="B156" s="59" t="inlineStr">
@@ -14311,7 +14306,7 @@
     <row r="157" ht="23.85" customHeight="1" s="36">
       <c r="A157" s="59" t="inlineStr">
         <is>
-          <t>AUT-029</t>
+          <t>AUT-023</t>
         </is>
       </c>
       <c r="B157" s="59" t="inlineStr">
@@ -14391,7 +14386,7 @@
     <row r="158" ht="23.85" customHeight="1" s="36">
       <c r="A158" s="59" t="inlineStr">
         <is>
-          <t>AUT-029</t>
+          <t>AUT-023</t>
         </is>
       </c>
       <c r="B158" s="59" t="inlineStr">
@@ -14467,7 +14462,7 @@
     <row r="159" ht="23.85" customHeight="1" s="36">
       <c r="A159" s="59" t="inlineStr">
         <is>
-          <t>AUT-029</t>
+          <t>AUT-023</t>
         </is>
       </c>
       <c r="B159" s="59" t="inlineStr">
@@ -14543,7 +14538,7 @@
     <row r="160" ht="23.85" customHeight="1" s="36">
       <c r="A160" s="49" t="inlineStr">
         <is>
-          <t>AUT-030</t>
+          <t>AUT-024</t>
         </is>
       </c>
       <c r="B160" s="49" t="inlineStr">
@@ -14623,7 +14618,7 @@
     <row r="161" ht="23.85" customHeight="1" s="36">
       <c r="A161" s="49" t="inlineStr">
         <is>
-          <t>AUT-030</t>
+          <t>AUT-024</t>
         </is>
       </c>
       <c r="B161" s="49" t="inlineStr">
@@ -14703,7 +14698,7 @@
     <row r="162" ht="23.85" customHeight="1" s="36">
       <c r="A162" s="49" t="inlineStr">
         <is>
-          <t>AUT-030</t>
+          <t>AUT-024</t>
         </is>
       </c>
       <c r="B162" s="49" t="inlineStr">
@@ -14783,7 +14778,7 @@
     <row r="163" ht="23.85" customHeight="1" s="36">
       <c r="A163" s="49" t="inlineStr">
         <is>
-          <t>AUT-030</t>
+          <t>AUT-024</t>
         </is>
       </c>
       <c r="B163" s="49" t="inlineStr">
@@ -14859,7 +14854,7 @@
     <row r="164" ht="23.85" customHeight="1" s="36">
       <c r="A164" s="49" t="inlineStr">
         <is>
-          <t>AUT-030</t>
+          <t>AUT-024</t>
         </is>
       </c>
       <c r="B164" s="49" t="inlineStr">
@@ -14935,7 +14930,7 @@
     <row r="165" ht="23.85" customHeight="1" s="36">
       <c r="A165" s="49" t="inlineStr">
         <is>
-          <t>AUT-030</t>
+          <t>AUT-024</t>
         </is>
       </c>
       <c r="B165" s="49" t="inlineStr">
@@ -15011,7 +15006,7 @@
     <row r="166" ht="15" customHeight="1" s="36">
       <c r="A166" s="59" t="inlineStr">
         <is>
-          <t>AUT-031</t>
+          <t>AUT-025</t>
         </is>
       </c>
       <c r="B166" s="59" t="inlineStr">
@@ -15091,7 +15086,7 @@
     <row r="167" ht="15" customHeight="1" s="36">
       <c r="A167" s="59" t="inlineStr">
         <is>
-          <t>AUT-031</t>
+          <t>AUT-025</t>
         </is>
       </c>
       <c r="B167" s="59" t="inlineStr">
@@ -15171,7 +15166,7 @@
     <row r="168" ht="15" customHeight="1" s="36">
       <c r="A168" s="59" t="inlineStr">
         <is>
-          <t>AUT-031</t>
+          <t>AUT-025</t>
         </is>
       </c>
       <c r="B168" s="59" t="inlineStr">
@@ -15251,7 +15246,7 @@
     <row r="169" ht="15" customHeight="1" s="36">
       <c r="A169" s="59" t="inlineStr">
         <is>
-          <t>AUT-031</t>
+          <t>AUT-025</t>
         </is>
       </c>
       <c r="B169" s="59" t="inlineStr">
@@ -15327,7 +15322,7 @@
     <row r="170" ht="15" customHeight="1" s="36">
       <c r="A170" s="59" t="inlineStr">
         <is>
-          <t>AUT-031</t>
+          <t>AUT-025</t>
         </is>
       </c>
       <c r="B170" s="59" t="inlineStr">
@@ -15407,7 +15402,7 @@
     <row r="171" ht="15" customHeight="1" s="36">
       <c r="A171" s="59" t="inlineStr">
         <is>
-          <t>AUT-031</t>
+          <t>AUT-025</t>
         </is>
       </c>
       <c r="B171" s="59" t="inlineStr">
@@ -15483,7 +15478,7 @@
     <row r="172" ht="15" customHeight="1" s="36">
       <c r="A172" s="59" t="inlineStr">
         <is>
-          <t>AUT-031</t>
+          <t>AUT-025</t>
         </is>
       </c>
       <c r="B172" s="59" t="inlineStr">
@@ -15563,7 +15558,7 @@
     <row r="173" ht="23.85" customHeight="1" s="36">
       <c r="A173" s="59" t="inlineStr">
         <is>
-          <t>AUT-031</t>
+          <t>AUT-025</t>
         </is>
       </c>
       <c r="B173" s="59" t="inlineStr">
@@ -15639,7 +15634,7 @@
     <row r="174" ht="15" customHeight="1" s="36">
       <c r="A174" s="49" t="inlineStr">
         <is>
-          <t>AUT-032</t>
+          <t>AUT-026</t>
         </is>
       </c>
       <c r="B174" s="49" t="inlineStr">
@@ -15719,7 +15714,7 @@
     <row r="175" ht="15" customHeight="1" s="36">
       <c r="A175" s="49" t="inlineStr">
         <is>
-          <t>AUT-032</t>
+          <t>AUT-026</t>
         </is>
       </c>
       <c r="B175" s="49" t="inlineStr">
@@ -15799,7 +15794,7 @@
     <row r="176" ht="15" customHeight="1" s="36">
       <c r="A176" s="49" t="inlineStr">
         <is>
-          <t>AUT-032</t>
+          <t>AUT-026</t>
         </is>
       </c>
       <c r="B176" s="49" t="inlineStr">
@@ -15879,7 +15874,7 @@
     <row r="177" ht="15" customHeight="1" s="36">
       <c r="A177" s="49" t="inlineStr">
         <is>
-          <t>AUT-032</t>
+          <t>AUT-026</t>
         </is>
       </c>
       <c r="B177" s="49" t="inlineStr">
@@ -15955,7 +15950,7 @@
     <row r="178" ht="15" customHeight="1" s="36">
       <c r="A178" s="49" t="inlineStr">
         <is>
-          <t>AUT-032</t>
+          <t>AUT-026</t>
         </is>
       </c>
       <c r="B178" s="49" t="inlineStr">
@@ -16031,7 +16026,7 @@
     <row r="179" ht="15" customHeight="1" s="36">
       <c r="A179" s="49" t="inlineStr">
         <is>
-          <t>AUT-032</t>
+          <t>AUT-026</t>
         </is>
       </c>
       <c r="B179" s="49" t="inlineStr">
@@ -16305,7 +16300,7 @@
     <row r="3" ht="15" customHeight="1" s="36">
       <c r="A3" s="49" t="inlineStr">
         <is>
-          <t>AUT-003</t>
+          <t>AUT-002</t>
         </is>
       </c>
       <c r="B3" s="41" t="inlineStr">
@@ -16353,7 +16348,7 @@
     <row r="4" ht="15" customHeight="1" s="36">
       <c r="A4" s="49" t="inlineStr">
         <is>
-          <t>AUT-004</t>
+          <t>AUT-003</t>
         </is>
       </c>
       <c r="B4" s="41" t="inlineStr">
@@ -16401,7 +16396,7 @@
     <row r="5" ht="15" customHeight="1" s="36">
       <c r="A5" s="49" t="inlineStr">
         <is>
-          <t>AUT-007</t>
+          <t>AUT-004</t>
         </is>
       </c>
       <c r="B5" s="41" t="inlineStr">
@@ -16449,7 +16444,7 @@
     <row r="6" ht="15" customHeight="1" s="36">
       <c r="A6" s="49" t="inlineStr">
         <is>
-          <t>AUT-008</t>
+          <t>AUT-005</t>
         </is>
       </c>
       <c r="B6" s="41" t="inlineStr">
@@ -16497,7 +16492,7 @@
     <row r="7" ht="15" customHeight="1" s="36">
       <c r="A7" s="49" t="inlineStr">
         <is>
-          <t>AUT-009</t>
+          <t>AUT-006</t>
         </is>
       </c>
       <c r="B7" s="41" t="inlineStr">
@@ -16545,7 +16540,7 @@
     <row r="8" ht="15" customHeight="1" s="36">
       <c r="A8" s="49" t="inlineStr">
         <is>
-          <t>AUT-010</t>
+          <t>AUT-007</t>
         </is>
       </c>
       <c r="B8" s="41" t="inlineStr">
@@ -16593,7 +16588,7 @@
     <row r="9" ht="15" customHeight="1" s="36">
       <c r="A9" s="49" t="inlineStr">
         <is>
-          <t>AUT-011</t>
+          <t>AUT-008</t>
         </is>
       </c>
       <c r="B9" s="41" t="inlineStr">
@@ -16641,7 +16636,7 @@
     <row r="10" ht="15" customHeight="1" s="36">
       <c r="A10" s="49" t="inlineStr">
         <is>
-          <t>AUT-012</t>
+          <t>AUT-009</t>
         </is>
       </c>
       <c r="B10" s="41" t="inlineStr">
@@ -16689,7 +16684,7 @@
     <row r="11" ht="15" customHeight="1" s="36">
       <c r="A11" s="49" t="inlineStr">
         <is>
-          <t>AUT-015</t>
+          <t>AUT-010</t>
         </is>
       </c>
       <c r="B11" s="41" t="inlineStr">
@@ -16737,7 +16732,7 @@
     <row r="12" ht="15" customHeight="1" s="36">
       <c r="A12" s="49" t="inlineStr">
         <is>
-          <t>AUT-016</t>
+          <t>AUT-011</t>
         </is>
       </c>
       <c r="B12" s="41" t="inlineStr">
@@ -16785,7 +16780,7 @@
     <row r="13" ht="15" customHeight="1" s="36">
       <c r="A13" s="49" t="inlineStr">
         <is>
-          <t>AUT-017</t>
+          <t>AUT-012</t>
         </is>
       </c>
       <c r="B13" s="41" t="inlineStr">
@@ -16833,7 +16828,7 @@
     <row r="14" ht="15" customHeight="1" s="36">
       <c r="A14" s="49" t="inlineStr">
         <is>
-          <t>AUT-018</t>
+          <t>AUT-013</t>
         </is>
       </c>
       <c r="B14" s="41" t="inlineStr">
@@ -16881,7 +16876,7 @@
     <row r="15" ht="15" customHeight="1" s="36">
       <c r="A15" s="49" t="inlineStr">
         <is>
-          <t>AUT-019</t>
+          <t>AUT-014</t>
         </is>
       </c>
       <c r="B15" s="41" t="inlineStr">
@@ -16929,7 +16924,7 @@
     <row r="16" ht="15" customHeight="1" s="36">
       <c r="A16" s="49" t="inlineStr">
         <is>
-          <t>AUT-021</t>
+          <t>AUT-015</t>
         </is>
       </c>
       <c r="B16" s="41" t="inlineStr">
@@ -16977,7 +16972,7 @@
     <row r="17" ht="15" customHeight="1" s="36">
       <c r="A17" s="49" t="inlineStr">
         <is>
-          <t>AUT-022</t>
+          <t>AUT-016</t>
         </is>
       </c>
       <c r="B17" s="41" t="inlineStr">
@@ -17025,7 +17020,7 @@
     <row r="18" ht="15" customHeight="1" s="36">
       <c r="A18" s="49" t="inlineStr">
         <is>
-          <t>AUT-023</t>
+          <t>AUT-017</t>
         </is>
       </c>
       <c r="B18" s="41" t="inlineStr">
@@ -17073,7 +17068,7 @@
     <row r="19" ht="15" customHeight="1" s="36">
       <c r="A19" s="49" t="inlineStr">
         <is>
-          <t>AUT-024</t>
+          <t>AUT-018</t>
         </is>
       </c>
       <c r="B19" s="41" t="inlineStr">
@@ -17121,7 +17116,7 @@
     <row r="20" ht="15" customHeight="1" s="36">
       <c r="A20" s="49" t="inlineStr">
         <is>
-          <t>AUT-025</t>
+          <t>AUT-019</t>
         </is>
       </c>
       <c r="B20" s="41" t="inlineStr">
@@ -17169,7 +17164,7 @@
     <row r="21" ht="15" customHeight="1" s="36">
       <c r="A21" s="49" t="inlineStr">
         <is>
-          <t>AUT-026</t>
+          <t>AUT-020</t>
         </is>
       </c>
       <c r="B21" s="41" t="inlineStr">
@@ -17217,7 +17212,7 @@
     <row r="22" ht="15" customHeight="1" s="36">
       <c r="A22" s="49" t="inlineStr">
         <is>
-          <t>AUT-027</t>
+          <t>AUT-021</t>
         </is>
       </c>
       <c r="B22" s="41" t="inlineStr">
@@ -17265,7 +17260,7 @@
     <row r="23" ht="15" customHeight="1" s="36">
       <c r="A23" s="49" t="inlineStr">
         <is>
-          <t>AUT-028</t>
+          <t>AUT-022</t>
         </is>
       </c>
       <c r="B23" s="41" t="inlineStr">
@@ -17313,7 +17308,7 @@
     <row r="24" ht="15" customHeight="1" s="36">
       <c r="A24" s="49" t="inlineStr">
         <is>
-          <t>AUT-029</t>
+          <t>AUT-023</t>
         </is>
       </c>
       <c r="B24" s="41" t="inlineStr">
@@ -17361,7 +17356,7 @@
     <row r="25" ht="23.85" customHeight="1" s="36">
       <c r="A25" s="49" t="inlineStr">
         <is>
-          <t>AUT-030</t>
+          <t>AUT-024</t>
         </is>
       </c>
       <c r="B25" s="41" t="inlineStr">
@@ -17409,7 +17404,7 @@
     <row r="26" ht="15" customHeight="1" s="36">
       <c r="A26" s="49" t="inlineStr">
         <is>
-          <t>AUT-031</t>
+          <t>AUT-025</t>
         </is>
       </c>
       <c r="B26" s="41" t="inlineStr">
@@ -17457,7 +17452,7 @@
     <row r="27" ht="15" customHeight="1" s="36">
       <c r="A27" s="49" t="inlineStr">
         <is>
-          <t>AUT-032</t>
+          <t>AUT-026</t>
         </is>
       </c>
       <c r="B27" s="41" t="inlineStr">
@@ -17659,7 +17654,7 @@
       </c>
       <c r="C2" s="49" t="inlineStr">
         <is>
-          <t>AUT-016</t>
+          <t>AUT-011</t>
         </is>
       </c>
       <c r="D2" s="49" t="inlineStr">
@@ -17727,7 +17722,7 @@
       </c>
       <c r="C3" s="49" t="inlineStr">
         <is>
-          <t>AUT-017</t>
+          <t>AUT-012</t>
         </is>
       </c>
       <c r="D3" s="49" t="inlineStr">
@@ -17795,7 +17790,7 @@
       </c>
       <c r="C4" s="49" t="inlineStr">
         <is>
-          <t>AUT-018</t>
+          <t>AUT-013</t>
         </is>
       </c>
       <c r="D4" s="49" t="inlineStr">
@@ -17863,7 +17858,7 @@
       </c>
       <c r="C5" s="49" t="inlineStr">
         <is>
-          <t>AUT-019</t>
+          <t>AUT-014</t>
         </is>
       </c>
       <c r="D5" s="49" t="inlineStr">
@@ -17999,7 +17994,7 @@
       </c>
       <c r="C7" s="49" t="inlineStr">
         <is>
-          <t>AUT-021</t>
+          <t>AUT-015</t>
         </is>
       </c>
       <c r="D7" s="49" t="inlineStr">
@@ -18135,7 +18130,7 @@
       </c>
       <c r="C9" s="49" t="inlineStr">
         <is>
-          <t>AUT-023</t>
+          <t>AUT-017</t>
         </is>
       </c>
       <c r="D9" s="49" t="inlineStr">
@@ -18203,7 +18198,7 @@
       </c>
       <c r="C10" s="49" t="inlineStr">
         <is>
-          <t>AUT-015, AUT-024</t>
+          <t>AUT-010, AUT-018</t>
         </is>
       </c>
       <c r="D10" s="49" t="inlineStr">
@@ -18271,7 +18266,7 @@
       </c>
       <c r="C11" s="49" t="inlineStr">
         <is>
-          <t>AUT-025</t>
+          <t>AUT-019</t>
         </is>
       </c>
       <c r="D11" s="49" t="inlineStr">
@@ -18339,7 +18334,7 @@
       </c>
       <c r="C12" s="49" t="inlineStr">
         <is>
-          <t>AUT-027</t>
+          <t>AUT-021</t>
         </is>
       </c>
       <c r="D12" s="49" t="inlineStr">
@@ -18407,7 +18402,7 @@
       </c>
       <c r="C13" s="49" t="inlineStr">
         <is>
-          <t>AUT-028</t>
+          <t>AUT-022</t>
         </is>
       </c>
       <c r="D13" s="49" t="inlineStr">
@@ -18475,7 +18470,7 @@
       </c>
       <c r="C14" s="49" t="inlineStr">
         <is>
-          <t>AUT-029</t>
+          <t>AUT-023</t>
         </is>
       </c>
       <c r="D14" s="49" t="inlineStr">
@@ -18543,7 +18538,7 @@
       </c>
       <c r="C15" s="49" t="inlineStr">
         <is>
-          <t>AUT-031</t>
+          <t>AUT-025</t>
         </is>
       </c>
       <c r="D15" s="49" t="inlineStr">
@@ -18611,7 +18606,7 @@
       </c>
       <c r="C16" s="49" t="inlineStr">
         <is>
-          <t>AUT-032</t>
+          <t>AUT-026</t>
         </is>
       </c>
       <c r="D16" s="49" t="inlineStr">
@@ -18679,7 +18674,7 @@
       </c>
       <c r="C17" s="49" t="inlineStr">
         <is>
-          <t>AUT-022</t>
+          <t>AUT-016</t>
         </is>
       </c>
       <c r="D17" s="49" t="inlineStr">
@@ -18747,7 +18742,7 @@
       </c>
       <c r="C18" s="49" t="inlineStr">
         <is>
-          <t>AUT-026</t>
+          <t>AUT-020</t>
         </is>
       </c>
       <c r="D18" s="49" t="inlineStr">
@@ -18815,7 +18810,7 @@
       </c>
       <c r="C19" s="49" t="inlineStr">
         <is>
-          <t>AUT-030</t>
+          <t>AUT-024</t>
         </is>
       </c>
       <c r="D19" s="49" t="inlineStr">

</xml_diff>